<commit_message>
generating week 7 queries (2/2).
</commit_message>
<xml_diff>
--- a/Function 5/evals.xlsx
+++ b/Function 5/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F784F9A1-02CD-4DC3-B5E3-889C8721B06A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A085E4-B615-43AD-8BE8-779D0FF6A253}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -543,7 +543,7 @@
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="2">
-        <v>0.86047684710456096</v>
+        <v>0.98399754414351104</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2">
@@ -647,26 +647,40 @@
     </row>
   </sheetData>
   <mergeCells count="66">
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="H9:I9"/>
@@ -679,40 +693,26 @@
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
generating week 9 queries (/2/2).
</commit_message>
<xml_diff>
--- a/Function 5/evals.xlsx
+++ b/Function 5/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2614661-034C-46BD-8C37-D7C1E97B8A8D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787A6C96-2A45-4C7B-8F05-713DBAAA7317}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -379,9 +379,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:M14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -407,7 +407,7 @@
       </c>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -433,7 +433,7 @@
       </c>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -459,7 +459,7 @@
       </c>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -485,7 +485,7 @@
       </c>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
         <v>4</v>
       </c>
@@ -511,7 +511,7 @@
       </c>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -537,7 +537,7 @@
       </c>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -563,7 +563,7 @@
       </c>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -584,24 +584,36 @@
         <v>1</v>
       </c>
       <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
+      <c r="L9" s="2">
+        <v>8662.4825000000001</v>
+      </c>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="3">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
       <c r="I10" s="2"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="J10" s="2">
+        <v>0.816851271636303</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -615,7 +627,7 @@
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -629,7 +641,7 @@
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -643,7 +655,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -658,19 +670,51 @@
       <c r="M14" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="68">
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
+  <mergeCells count="70">
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
@@ -683,50 +727,20 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="J10:K10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>